<commit_message>
Update Bạch Mai Thiên Tú (Thôn Đầm Rải): add class/school, fix birth year
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -11229,7 +11229,11 @@
           <t>Bạch Mai Thiên Tú</t>
         </is>
       </c>
-      <c r="C898" s="30" t="inlineStr"/>
+      <c r="C898" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 6 - TH&amp;THCS Nhuận Trạch</t>
+        </is>
+      </c>
       <c r="D898" s="31" t="inlineStr">
         <is>
           <t>Thôn Đầm Rải</t>
@@ -11243,7 +11247,7 @@
       <c r="F898" s="31" t="inlineStr"/>
       <c r="G898" s="32" t="inlineStr">
         <is>
-          <t>SN: 17/11/2021</t>
+          <t>SN: 17/11/2014</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 3 children to Thôn Giếng Êm; consolidate TK12 and Đầm Rải edits
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -2321,14 +2321,14 @@
       </c>
       <c r="E54" s="8" t="inlineStr"/>
       <c r="F54" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="G54" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="G54" s="39" t="n">
-        <v>3</v>
-      </c>
       <c r="H54" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>✅ Đủ DS</t>
         </is>
       </c>
     </row>
@@ -12492,46 +12492,94 @@
       <c r="A1024" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B1024" s="19" t="inlineStr"/>
-      <c r="C1024" s="20" t="inlineStr"/>
+      <c r="B1024" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Tiến Mạnh</t>
+        </is>
+      </c>
+      <c r="C1024" s="20" t="inlineStr">
+        <is>
+          <t>MN Nhuận Trạch</t>
+        </is>
+      </c>
       <c r="D1024" s="21" t="inlineStr">
         <is>
           <t>Thôn Giếng Êm</t>
         </is>
       </c>
-      <c r="E1024" s="20" t="inlineStr"/>
+      <c r="E1024" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F1024" s="21" t="inlineStr"/>
-      <c r="G1024" s="22" t="inlineStr"/>
+      <c r="G1024" s="22" t="inlineStr">
+        <is>
+          <t>SN: 06/12/2020</t>
+        </is>
+      </c>
     </row>
     <row r="1025" ht="22" customHeight="1">
       <c r="A1025" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B1025" s="19" t="inlineStr"/>
-      <c r="C1025" s="20" t="inlineStr"/>
+      <c r="B1025" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Ngọc Châm</t>
+        </is>
+      </c>
+      <c r="C1025" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Nhuận Trạch</t>
+        </is>
+      </c>
       <c r="D1025" s="21" t="inlineStr">
         <is>
           <t>Thôn Giếng Êm</t>
         </is>
       </c>
-      <c r="E1025" s="20" t="inlineStr"/>
+      <c r="E1025" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F1025" s="21" t="inlineStr"/>
-      <c r="G1025" s="22" t="inlineStr"/>
+      <c r="G1025" s="22" t="inlineStr">
+        <is>
+          <t>SN: 15/07/2015</t>
+        </is>
+      </c>
     </row>
     <row r="1026" ht="22" customHeight="1">
       <c r="A1026" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B1026" s="19" t="inlineStr"/>
-      <c r="C1026" s="20" t="inlineStr"/>
+      <c r="B1026" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Minh Tâm</t>
+        </is>
+      </c>
+      <c r="C1026" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Nhuận Trạch</t>
+        </is>
+      </c>
       <c r="D1026" s="21" t="inlineStr">
         <is>
           <t>Thôn Giếng Êm</t>
         </is>
       </c>
-      <c r="E1026" s="20" t="inlineStr"/>
+      <c r="E1026" s="20" t="inlineStr">
+        <is>
+          <t>Khuyết tật</t>
+        </is>
+      </c>
       <c r="F1026" s="21" t="inlineStr"/>
-      <c r="G1026" s="22" t="inlineStr"/>
+      <c r="G1026" s="22" t="inlineStr">
+        <is>
+          <t>SN: 28/10/2014</t>
+        </is>
+      </c>
     </row>
     <row r="1027" ht="16" customHeight="1">
       <c r="A1027" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Add children to multiple hamlets (file list + TK11/TK12/Bằng Gà/Cột Bài/Thầy Mò)
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -819,14 +819,14 @@
         </is>
       </c>
       <c r="F5" s="39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H5" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>⏳ Còn thiếu 3</t>
         </is>
       </c>
     </row>
@@ -1003,14 +1003,14 @@
       </c>
       <c r="E11" s="8" t="inlineStr"/>
       <c r="F11" s="39" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="39" t="n">
-        <v>3</v>
-      </c>
       <c r="H11" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>⚠️ Vượt 1</t>
         </is>
       </c>
     </row>
@@ -1033,14 +1033,14 @@
       </c>
       <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G12" s="39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H12" s="40" t="inlineStr">
         <is>
-          <t>⏳ Còn thiếu 2</t>
+          <t>⚠️ Vượt 1</t>
         </is>
       </c>
     </row>
@@ -1191,14 +1191,14 @@
         </is>
       </c>
       <c r="F17" s="39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" s="39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H17" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>⏳ Còn thiếu 2</t>
         </is>
       </c>
     </row>
@@ -1469,14 +1469,14 @@
         </is>
       </c>
       <c r="F26" s="41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G26" s="41" t="n">
         <v>0</v>
       </c>
       <c r="H26" s="42" t="inlineStr">
         <is>
-          <t>✅ Đủ DS</t>
+          <t>⚠️ Vượt 1</t>
         </is>
       </c>
     </row>
@@ -1503,14 +1503,14 @@
         </is>
       </c>
       <c r="F27" s="39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G27" s="39" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H27" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>⏳ Còn thiếu 4</t>
         </is>
       </c>
     </row>
@@ -1537,14 +1537,14 @@
         </is>
       </c>
       <c r="F28" s="39" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="39" t="n">
-        <v>5</v>
-      </c>
       <c r="H28" s="40" t="inlineStr">
         <is>
-          <t>⛔ Chưa gửi DS</t>
+          <t>✅ Đủ DS</t>
         </is>
       </c>
     </row>
@@ -1571,14 +1571,14 @@
         </is>
       </c>
       <c r="F29" s="41" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G29" s="41" t="n">
         <v>0</v>
       </c>
       <c r="H29" s="42" t="inlineStr">
         <is>
-          <t>✅ Đủ DS</t>
+          <t>⚠️ Vượt 3</t>
         </is>
       </c>
     </row>
@@ -2572,16 +2572,32 @@
       <c r="A7" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="19" t="inlineStr"/>
-      <c r="C7" s="20" t="inlineStr"/>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Trang Dung</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 2</t>
         </is>
       </c>
-      <c r="E7" s="20" t="inlineStr"/>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Hộ cận nghèo đơn thân, mẹ bệnh tật không có việc làm, cháu là TEKT</t>
+        </is>
+      </c>
       <c r="F7" s="21" t="inlineStr"/>
-      <c r="G7" s="22" t="inlineStr"/>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>SN: 27/08/2015</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="18" t="n">
@@ -3805,88 +3821,169 @@
       <c r="A128" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B128" s="19" t="inlineStr"/>
-      <c r="C128" s="20" t="inlineStr"/>
+      <c r="B128" s="19" t="inlineStr">
+        <is>
+          <t>Vương Nhật Khang</t>
+        </is>
+      </c>
+      <c r="C128" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Cửu Long</t>
+        </is>
+      </c>
       <c r="D128" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 11</t>
         </is>
       </c>
-      <c r="E128" s="20" t="inlineStr"/>
+      <c r="E128" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F128" s="21" t="inlineStr"/>
-      <c r="G128" s="22" t="inlineStr"/>
+      <c r="G128" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2015</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="22" customHeight="1">
       <c r="A129" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B129" s="19" t="inlineStr"/>
-      <c r="C129" s="20" t="inlineStr"/>
+      <c r="B129" s="19" t="inlineStr">
+        <is>
+          <t>Vũ Đức Đam</t>
+        </is>
+      </c>
+      <c r="C129" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 7 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D129" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 11</t>
         </is>
       </c>
-      <c r="E129" s="20" t="inlineStr"/>
+      <c r="E129" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F129" s="21" t="inlineStr"/>
-      <c r="G129" s="22" t="inlineStr"/>
+      <c r="G129" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2013</t>
+        </is>
+      </c>
     </row>
     <row r="130" ht="22" customHeight="1">
       <c r="A130" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B130" s="19" t="inlineStr"/>
-      <c r="C130" s="20" t="inlineStr"/>
+      <c r="B130" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Khải Anh</t>
+        </is>
+      </c>
+      <c r="C130" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 2 - TH&amp;THCS Cửu Long</t>
+        </is>
+      </c>
       <c r="D130" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 11</t>
         </is>
       </c>
-      <c r="E130" s="20" t="inlineStr"/>
+      <c r="E130" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F130" s="21" t="inlineStr"/>
-      <c r="G130" s="22" t="inlineStr"/>
+      <c r="G130" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2018</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="16" customHeight="1">
-      <c r="A131" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 03 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="8" customHeight="1"/>
+      <c r="A131" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B131" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Hà Linh</t>
+        </is>
+      </c>
+      <c r="C131" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 2 - TH&amp;THCS Cửu Long</t>
+        </is>
+      </c>
+      <c r="D131" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu 11</t>
+        </is>
+      </c>
+      <c r="E131" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F131" s="21" t="n"/>
+      <c r="G131" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2018</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="8" customHeight="1">
+      <c r="A132" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 04 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="133" ht="8" customHeight="1"/>
     <row r="134" ht="16" customHeight="1">
-      <c r="D134" s="24" t="inlineStr">
+      <c r="D134" s="24" t="n"/>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="25" t="n"/>
+      <c r="D135" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="25" t="inlineStr">
+    <row r="136" ht="16" customHeight="1">
+      <c r="A136" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E135" s="25" t="inlineStr">
+      <c r="E136" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="136" ht="16" customHeight="1">
-      <c r="A136" s="26" t="inlineStr">
+    <row r="137" ht="6" customHeight="1">
+      <c r="A137" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E136" s="26" t="inlineStr">
+      <c r="E137" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="137" ht="6" customHeight="1"/>
     <row r="138" ht="6" customHeight="1"/>
     <row r="139" ht="6" customHeight="1"/>
     <row r="140" ht="4" customHeight="1">
@@ -3898,7 +3995,15 @@
       <c r="F140" s="27" t="n"/>
       <c r="G140" s="27" t="n"/>
     </row>
-    <row r="141" ht="6" customHeight="1"/>
+    <row r="141" ht="6" customHeight="1">
+      <c r="A141" s="27" t="n"/>
+      <c r="B141" s="27" t="n"/>
+      <c r="C141" s="27" t="n"/>
+      <c r="D141" s="27" t="n"/>
+      <c r="E141" s="27" t="n"/>
+      <c r="F141" s="27" t="n"/>
+      <c r="G141" s="27" t="n"/>
+    </row>
     <row r="142" ht="14" customHeight="1">
       <c r="G142" s="14" t="inlineStr">
         <is>
@@ -3972,10 +4077,14 @@
       </c>
       <c r="B148" s="19" t="inlineStr">
         <is>
-          <t>Nguyễn Khắc Kim Anh</t>
-        </is>
-      </c>
-      <c r="C148" s="20" t="inlineStr"/>
+          <t>Nguyễn Tuệ Lâm</t>
+        </is>
+      </c>
+      <c r="C148" s="20" t="inlineStr">
+        <is>
+          <t>Mầm non</t>
+        </is>
+      </c>
       <c r="D148" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 12</t>
@@ -3983,13 +4092,13 @@
       </c>
       <c r="E148" s="20" t="inlineStr">
         <is>
-          <t>Hộ khó khăn</t>
+          <t>Hộ khó khăn (không có bố)</t>
         </is>
       </c>
       <c r="F148" s="21" t="inlineStr"/>
       <c r="G148" s="22" t="inlineStr">
         <is>
-          <t>SN: 30/06/2013</t>
+          <t>SN: 2020</t>
         </is>
       </c>
     </row>
@@ -3997,73 +4106,134 @@
       <c r="A149" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B149" s="19" t="inlineStr"/>
-      <c r="C149" s="20" t="inlineStr"/>
+      <c r="B149" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Ngọc Thiên Anh</t>
+        </is>
+      </c>
+      <c r="C149" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5</t>
+        </is>
+      </c>
       <c r="D149" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 12</t>
         </is>
       </c>
-      <c r="E149" s="20" t="inlineStr"/>
+      <c r="E149" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn (không có mẹ)</t>
+        </is>
+      </c>
       <c r="F149" s="21" t="inlineStr"/>
-      <c r="G149" s="22" t="inlineStr"/>
+      <c r="G149" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2015</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="22" customHeight="1">
       <c r="A150" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B150" s="19" t="inlineStr"/>
-      <c r="C150" s="20" t="inlineStr"/>
+      <c r="B150" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Khắc Kim Anh</t>
+        </is>
+      </c>
+      <c r="C150" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 7</t>
+        </is>
+      </c>
       <c r="D150" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 12</t>
         </is>
       </c>
-      <c r="E150" s="20" t="inlineStr"/>
+      <c r="E150" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn (không có bố)</t>
+        </is>
+      </c>
       <c r="F150" s="21" t="inlineStr"/>
-      <c r="G150" s="22" t="inlineStr"/>
+      <c r="G150" s="22" t="inlineStr">
+        <is>
+          <t>SN: 30/06/2013</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="16" customHeight="1">
-      <c r="A151" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 03 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="8" customHeight="1"/>
+      <c r="A151" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B151" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Bá Đạt</t>
+        </is>
+      </c>
+      <c r="C151" s="20" t="inlineStr"/>
+      <c r="D151" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu 12</t>
+        </is>
+      </c>
+      <c r="E151" s="20" t="inlineStr">
+        <is>
+          <t>Khuyết tật, hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F151" s="21" t="n"/>
+      <c r="G151" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2006</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="8" customHeight="1">
+      <c r="A152" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 04 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="153" ht="8" customHeight="1"/>
     <row r="154" ht="16" customHeight="1">
-      <c r="D154" s="24" t="inlineStr">
+      <c r="D154" s="24" t="n"/>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="25" t="n"/>
+      <c r="D155" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="155" ht="18" customHeight="1">
-      <c r="A155" s="25" t="inlineStr">
+    <row r="156" ht="16" customHeight="1">
+      <c r="A156" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E155" s="25" t="inlineStr">
+      <c r="E156" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="16" customHeight="1">
-      <c r="A156" s="26" t="inlineStr">
+    <row r="157" ht="6" customHeight="1">
+      <c r="A157" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E156" s="26" t="inlineStr">
+      <c r="E157" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="6" customHeight="1"/>
     <row r="158" ht="6" customHeight="1"/>
     <row r="159" ht="6" customHeight="1"/>
     <row r="160" ht="4" customHeight="1">
@@ -4075,7 +4245,15 @@
       <c r="F160" s="27" t="n"/>
       <c r="G160" s="27" t="n"/>
     </row>
-    <row r="161" ht="6" customHeight="1"/>
+    <row r="161" ht="6" customHeight="1">
+      <c r="A161" s="27" t="n"/>
+      <c r="B161" s="27" t="n"/>
+      <c r="C161" s="27" t="n"/>
+      <c r="D161" s="27" t="n"/>
+      <c r="E161" s="27" t="n"/>
+      <c r="F161" s="27" t="n"/>
+      <c r="G161" s="27" t="n"/>
+    </row>
     <row r="162" ht="14" customHeight="1">
       <c r="G162" s="14" t="inlineStr">
         <is>
@@ -4524,7 +4702,7 @@
       </c>
       <c r="C208" s="30" t="inlineStr">
         <is>
-          <t>Lớp 6 - TH Hùng Sơn</t>
+          <t>Lớp 6 - TH&amp;THCS Hùng Sơn</t>
         </is>
       </c>
       <c r="D208" s="36" t="inlineStr">
@@ -4538,7 +4716,11 @@
         </is>
       </c>
       <c r="F208" s="36" t="inlineStr"/>
-      <c r="G208" s="33" t="inlineStr"/>
+      <c r="G208" s="33" t="inlineStr">
+        <is>
+          <t>SN: 04/10/2015</t>
+        </is>
+      </c>
     </row>
     <row r="209" ht="22" customHeight="1">
       <c r="A209" s="35" t="n">
@@ -4919,16 +5101,32 @@
       <c r="A248" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B248" s="19" t="inlineStr"/>
-      <c r="C248" s="20" t="inlineStr"/>
+      <c r="B248" s="19" t="inlineStr">
+        <is>
+          <t>Đinh Quỳnh Như</t>
+        </is>
+      </c>
+      <c r="C248" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D248" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu Mò</t>
         </is>
       </c>
-      <c r="E248" s="20" t="inlineStr"/>
+      <c r="E248" s="20" t="inlineStr">
+        <is>
+          <t>Hộ cận nghèo đơn thân, mẹ bệnh tật không có việc làm, cháu là TEKT</t>
+        </is>
+      </c>
       <c r="F248" s="21" t="inlineStr"/>
-      <c r="G248" s="22" t="inlineStr"/>
+      <c r="G248" s="22" t="inlineStr">
+        <is>
+          <t>SN: 21/01/2015</t>
+        </is>
+      </c>
     </row>
     <row r="249" ht="22" customHeight="1">
       <c r="A249" s="18" t="n">
@@ -6067,7 +6265,11 @@
           <t>Bùi Khánh Phương</t>
         </is>
       </c>
-      <c r="C371" s="30" t="inlineStr"/>
+      <c r="C371" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 3 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D371" s="31" t="inlineStr">
         <is>
           <t>Xóm Vẽ</t>
@@ -6075,11 +6277,15 @@
       </c>
       <c r="E371" s="30" t="inlineStr">
         <is>
-          <t>Hộ nghèo (đã có trong ds)</t>
+          <t>Hộ nghèo, mồ côi bố</t>
         </is>
       </c>
       <c r="F371" s="31" t="inlineStr"/>
-      <c r="G371" s="33" t="inlineStr"/>
+      <c r="G371" s="33" t="inlineStr">
+        <is>
+          <t>SN: 30/01/2017</t>
+        </is>
+      </c>
     </row>
     <row r="372" ht="22" customHeight="1">
       <c r="A372" s="28" t="n">
@@ -6943,46 +7149,79 @@
       <c r="G441" s="33" t="inlineStr"/>
     </row>
     <row r="442" ht="16" customHeight="1">
-      <c r="A442" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 05 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="443" ht="8" customHeight="1"/>
+      <c r="A442" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B442" s="29" t="inlineStr">
+        <is>
+          <t>Nguyễn Diệu Thuỳ</t>
+        </is>
+      </c>
+      <c r="C442" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 6 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
+      <c r="D442" s="31" t="inlineStr">
+        <is>
+          <t>Thầy Mò</t>
+        </is>
+      </c>
+      <c r="E442" s="30" t="inlineStr">
+        <is>
+          <t>Hộ nghèo, bố mẹ ly hôn</t>
+        </is>
+      </c>
+      <c r="F442" s="31" t="n"/>
+      <c r="G442" s="33" t="inlineStr">
+        <is>
+          <t>SN: 18/01/2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="443" ht="8" customHeight="1">
+      <c r="A443" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 06 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="444" ht="8" customHeight="1"/>
     <row r="445" ht="16" customHeight="1">
-      <c r="D445" s="24" t="inlineStr">
+      <c r="D445" s="24" t="n"/>
+    </row>
+    <row r="446" ht="18" customHeight="1">
+      <c r="A446" s="25" t="n"/>
+      <c r="D446" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="446" ht="18" customHeight="1">
-      <c r="A446" s="25" t="inlineStr">
+    <row r="447" ht="16" customHeight="1">
+      <c r="A447" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E446" s="25" t="inlineStr">
+      <c r="E447" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="447" ht="16" customHeight="1">
-      <c r="A447" s="26" t="inlineStr">
+    <row r="448" ht="6" customHeight="1">
+      <c r="A448" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E447" s="26" t="inlineStr">
+      <c r="E448" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="448" ht="6" customHeight="1"/>
     <row r="449" ht="6" customHeight="1"/>
     <row r="450" ht="6" customHeight="1"/>
     <row r="451" ht="4" customHeight="1">
@@ -6994,7 +7233,15 @@
       <c r="F451" s="27" t="n"/>
       <c r="G451" s="27" t="n"/>
     </row>
-    <row r="452" ht="6" customHeight="1"/>
+    <row r="452" ht="6" customHeight="1">
+      <c r="A452" s="27" t="n"/>
+      <c r="B452" s="27" t="n"/>
+      <c r="C452" s="27" t="n"/>
+      <c r="D452" s="27" t="n"/>
+      <c r="E452" s="27" t="n"/>
+      <c r="F452" s="27" t="n"/>
+      <c r="G452" s="27" t="n"/>
+    </row>
     <row r="453" ht="14" customHeight="1">
       <c r="G453" s="14" t="inlineStr">
         <is>
@@ -7066,16 +7313,32 @@
       <c r="A459" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B459" s="19" t="inlineStr"/>
-      <c r="C459" s="20" t="inlineStr"/>
+      <c r="B459" s="19" t="inlineStr">
+        <is>
+          <t>Hoàng Công Tuấn</t>
+        </is>
+      </c>
+      <c r="C459" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 8 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D459" s="21" t="inlineStr">
         <is>
           <t>Xóm Chanh</t>
         </is>
       </c>
-      <c r="E459" s="20" t="inlineStr"/>
+      <c r="E459" s="20" t="inlineStr">
+        <is>
+          <t>Hộ nghèo, mồ côi mẹ</t>
+        </is>
+      </c>
       <c r="F459" s="21" t="inlineStr"/>
-      <c r="G459" s="22" t="inlineStr"/>
+      <c r="G459" s="22" t="inlineStr">
+        <is>
+          <t>SN: 16/08/2012</t>
+        </is>
+      </c>
     </row>
     <row r="460" ht="22" customHeight="1">
       <c r="A460" s="18" t="n">
@@ -7261,76 +7524,156 @@
       <c r="A481" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="B481" s="19" t="inlineStr"/>
-      <c r="C481" s="20" t="inlineStr"/>
+      <c r="B481" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Thị Dung</t>
+        </is>
+      </c>
+      <c r="C481" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 8 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D481" s="21" t="inlineStr">
         <is>
           <t>Bằng Gà</t>
         </is>
       </c>
-      <c r="E481" s="20" t="inlineStr"/>
+      <c r="E481" s="20" t="inlineStr">
+        <is>
+          <t>Hộ nghèo có HCKK</t>
+        </is>
+      </c>
       <c r="F481" s="21" t="inlineStr"/>
-      <c r="G481" s="22" t="inlineStr"/>
+      <c r="G481" s="22" t="inlineStr">
+        <is>
+          <t>SN: 24/06/2012</t>
+        </is>
+      </c>
     </row>
     <row r="482" ht="22" customHeight="1">
       <c r="A482" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B482" s="19" t="inlineStr"/>
-      <c r="C482" s="20" t="inlineStr"/>
+      <c r="B482" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Thị Phương Thảo</t>
+        </is>
+      </c>
+      <c r="C482" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D482" s="21" t="inlineStr">
         <is>
           <t>Bằng Gà</t>
         </is>
       </c>
-      <c r="E482" s="20" t="inlineStr"/>
+      <c r="E482" s="20" t="inlineStr">
+        <is>
+          <t>Hộ nghèo có HCKK (đông con)</t>
+        </is>
+      </c>
       <c r="F482" s="21" t="inlineStr"/>
-      <c r="G482" s="22" t="inlineStr"/>
+      <c r="G482" s="22" t="inlineStr">
+        <is>
+          <t>SN: 29/10/2015</t>
+        </is>
+      </c>
     </row>
     <row r="483" ht="22" customHeight="1">
       <c r="A483" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B483" s="19" t="inlineStr"/>
-      <c r="C483" s="20" t="inlineStr"/>
+      <c r="B483" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Quỳnh Trang</t>
+        </is>
+      </c>
+      <c r="C483" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 3A2 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
       <c r="D483" s="21" t="inlineStr">
         <is>
           <t>Bằng Gà</t>
         </is>
       </c>
-      <c r="E483" s="20" t="inlineStr"/>
+      <c r="E483" s="20" t="inlineStr">
+        <is>
+          <t>Hộ nghèo</t>
+        </is>
+      </c>
       <c r="F483" s="21" t="inlineStr"/>
-      <c r="G483" s="22" t="inlineStr"/>
+      <c r="G483" s="22" t="inlineStr">
+        <is>
+          <t>SN: 17/12/2017</t>
+        </is>
+      </c>
     </row>
     <row r="484" ht="22" customHeight="1">
       <c r="A484" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B484" s="19" t="inlineStr"/>
-      <c r="C484" s="20" t="inlineStr"/>
+      <c r="B484" s="19" t="inlineStr">
+        <is>
+          <t>Hoàng Thế Khương</t>
+        </is>
+      </c>
+      <c r="C484" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 3A2 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
       <c r="D484" s="21" t="inlineStr">
         <is>
           <t>Bằng Gà</t>
         </is>
       </c>
-      <c r="E484" s="20" t="inlineStr"/>
+      <c r="E484" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F484" s="21" t="inlineStr"/>
-      <c r="G484" s="22" t="inlineStr"/>
+      <c r="G484" s="22" t="inlineStr">
+        <is>
+          <t>SN: 08/02/2017</t>
+        </is>
+      </c>
     </row>
     <row r="485" ht="22" customHeight="1">
       <c r="A485" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="B485" s="19" t="inlineStr"/>
-      <c r="C485" s="20" t="inlineStr"/>
+      <c r="B485" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Nam Thịnh</t>
+        </is>
+      </c>
+      <c r="C485" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 1 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
       <c r="D485" s="21" t="inlineStr">
         <is>
           <t>Bằng Gà</t>
         </is>
       </c>
-      <c r="E485" s="20" t="inlineStr"/>
+      <c r="E485" s="20" t="inlineStr">
+        <is>
+          <t>Hộ cận nghèo</t>
+        </is>
+      </c>
       <c r="F485" s="21" t="inlineStr"/>
-      <c r="G485" s="22" t="inlineStr"/>
+      <c r="G485" s="22" t="inlineStr">
+        <is>
+          <t>SN: 13/01/2019</t>
+        </is>
+      </c>
     </row>
     <row r="486" ht="16" customHeight="1">
       <c r="A486" s="23" t="inlineStr">
@@ -7461,7 +7804,11 @@
           <t>Bùi Quốc Khánh</t>
         </is>
       </c>
-      <c r="C503" s="30" t="inlineStr"/>
+      <c r="C503" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 2 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
       <c r="D503" s="31" t="inlineStr">
         <is>
           <t>Cột Bài</t>
@@ -7469,11 +7816,15 @@
       </c>
       <c r="E503" s="30" t="inlineStr">
         <is>
-          <t>Hộ nghèo (đã có trong ds)</t>
+          <t>Hộ nghèo, bố mẹ ly hôn</t>
         </is>
       </c>
       <c r="F503" s="31" t="inlineStr"/>
-      <c r="G503" s="33" t="inlineStr"/>
+      <c r="G503" s="33" t="inlineStr">
+        <is>
+          <t>SN: 03/09/2018</t>
+        </is>
+      </c>
     </row>
     <row r="504" ht="22" customHeight="1">
       <c r="A504" s="28" t="n">
@@ -7600,48 +7951,144 @@
       </c>
     </row>
     <row r="508" ht="16" customHeight="1">
-      <c r="A508" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 05 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="509" ht="8" customHeight="1"/>
-    <row r="510" ht="8" customHeight="1"/>
+      <c r="A508" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B508" s="29" t="inlineStr">
+        <is>
+          <t>Bùi Anh Tú</t>
+        </is>
+      </c>
+      <c r="C508" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 4 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
+      <c r="D508" s="31" t="inlineStr">
+        <is>
+          <t>Cột Bài</t>
+        </is>
+      </c>
+      <c r="E508" s="30" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F508" s="31" t="n"/>
+      <c r="G508" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="509" ht="8" customHeight="1">
+      <c r="A509" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="B509" s="29" t="inlineStr">
+        <is>
+          <t>Đinh Hồng Chinh</t>
+        </is>
+      </c>
+      <c r="C509" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 8 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
+      <c r="D509" s="31" t="inlineStr">
+        <is>
+          <t>Cột Bài</t>
+        </is>
+      </c>
+      <c r="E509" s="30" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F509" s="31" t="n"/>
+      <c r="G509" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="8" customHeight="1">
+      <c r="A510" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="B510" s="29" t="inlineStr">
+        <is>
+          <t>Đinh Thúy Hường</t>
+        </is>
+      </c>
+      <c r="C510" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 3 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
+      <c r="D510" s="31" t="inlineStr">
+        <is>
+          <t>Cột Bài</t>
+        </is>
+      </c>
+      <c r="E510" s="30" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F510" s="31" t="n"/>
+      <c r="G510" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2014</t>
+        </is>
+      </c>
+    </row>
     <row r="511" ht="16" customHeight="1">
-      <c r="D511" s="24" t="inlineStr">
+      <c r="A511" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 08 trẻ em.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="18" customHeight="1">
+      <c r="A512" s="25" t="n"/>
+      <c r="E512" s="25" t="n"/>
+    </row>
+    <row r="513" ht="16" customHeight="1">
+      <c r="A513" s="26" t="n"/>
+      <c r="E513" s="26" t="n"/>
+    </row>
+    <row r="514" ht="6" customHeight="1">
+      <c r="D514" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="512" ht="18" customHeight="1">
-      <c r="A512" s="25" t="inlineStr">
+    <row r="515" ht="6" customHeight="1">
+      <c r="A515" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E512" s="25" t="inlineStr">
+      <c r="E515" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="513" ht="16" customHeight="1">
-      <c r="A513" s="26" t="inlineStr">
+    <row r="516" ht="6" customHeight="1">
+      <c r="A516" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E513" s="26" t="inlineStr">
+      <c r="E516" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="514" ht="6" customHeight="1"/>
-    <row r="515" ht="6" customHeight="1"/>
-    <row r="516" ht="6" customHeight="1"/>
     <row r="517" ht="4" customHeight="1">
       <c r="A517" s="27" t="n"/>
       <c r="B517" s="27" t="n"/>
@@ -13358,7 +13805,6 @@
     <mergeCell ref="E381:G381"/>
     <mergeCell ref="A103:G103"/>
     <mergeCell ref="E16:G16"/>
-    <mergeCell ref="E512:G512"/>
     <mergeCell ref="E1052:G1052"/>
     <mergeCell ref="D254:G254"/>
     <mergeCell ref="A413:G413"/>
@@ -13372,7 +13818,6 @@
     <mergeCell ref="A479:G479"/>
     <mergeCell ref="A650:G650"/>
     <mergeCell ref="D114:G114"/>
-    <mergeCell ref="A131:G131"/>
     <mergeCell ref="A665:G665"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="E717:G717"/>
@@ -13396,6 +13841,7 @@
     <mergeCell ref="D489:G489"/>
     <mergeCell ref="E195:G195"/>
     <mergeCell ref="A358:C358"/>
+    <mergeCell ref="D135:G135"/>
     <mergeCell ref="E843:G843"/>
     <mergeCell ref="A4:G4"/>
     <mergeCell ref="E991:G991"/>
@@ -13410,7 +13856,6 @@
     <mergeCell ref="A1021:G1021"/>
     <mergeCell ref="A266:G266"/>
     <mergeCell ref="A215:C215"/>
-    <mergeCell ref="A513:C513"/>
     <mergeCell ref="D1112:G1112"/>
     <mergeCell ref="D1091:G1091"/>
     <mergeCell ref="E675:G675"/>
@@ -13423,8 +13868,9 @@
     <mergeCell ref="A749:G749"/>
     <mergeCell ref="A434:G434"/>
     <mergeCell ref="A1047:G1047"/>
+    <mergeCell ref="D446:G446"/>
     <mergeCell ref="A86:G86"/>
-    <mergeCell ref="A151:G151"/>
+    <mergeCell ref="A137:C137"/>
     <mergeCell ref="A572:C572"/>
     <mergeCell ref="A734:G734"/>
     <mergeCell ref="A864:C864"/>
@@ -13433,6 +13879,7 @@
     <mergeCell ref="A1093:C1093"/>
     <mergeCell ref="A671:G671"/>
     <mergeCell ref="A381:C381"/>
+    <mergeCell ref="A152:G152"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="A686:G686"/>
     <mergeCell ref="A76:C76"/>
@@ -13446,7 +13893,6 @@
     <mergeCell ref="A990:C990"/>
     <mergeCell ref="A292:G292"/>
     <mergeCell ref="A928:C928"/>
-    <mergeCell ref="D154:G154"/>
     <mergeCell ref="A286:G286"/>
     <mergeCell ref="A528:G528"/>
     <mergeCell ref="A851:G851"/>
@@ -13454,6 +13900,7 @@
     <mergeCell ref="A216:C216"/>
     <mergeCell ref="D632:G632"/>
     <mergeCell ref="A163:G163"/>
+    <mergeCell ref="A516:C516"/>
     <mergeCell ref="A316:C316"/>
     <mergeCell ref="A790:G790"/>
     <mergeCell ref="A895:G895"/>
@@ -13469,21 +13916,20 @@
     <mergeCell ref="A613:C613"/>
     <mergeCell ref="A45:G45"/>
     <mergeCell ref="A1042:G1042"/>
+    <mergeCell ref="D155:G155"/>
     <mergeCell ref="A623:G623"/>
     <mergeCell ref="A523:G523"/>
     <mergeCell ref="A345:G345"/>
     <mergeCell ref="E425:G425"/>
     <mergeCell ref="E696:G696"/>
-    <mergeCell ref="A446:C446"/>
     <mergeCell ref="A46:G46"/>
     <mergeCell ref="D905:G905"/>
     <mergeCell ref="E633:G633"/>
     <mergeCell ref="A105:G105"/>
     <mergeCell ref="A376:G376"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="E135:G135"/>
+    <mergeCell ref="D842:G842"/>
     <mergeCell ref="E35:G35"/>
-    <mergeCell ref="D842:G842"/>
     <mergeCell ref="E697:G697"/>
     <mergeCell ref="E802:G802"/>
     <mergeCell ref="A71:G71"/>
@@ -13518,12 +13964,12 @@
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="D926:G926"/>
+    <mergeCell ref="A448:C448"/>
     <mergeCell ref="A588:G588"/>
-    <mergeCell ref="A512:C512"/>
+    <mergeCell ref="E1031:G1031"/>
     <mergeCell ref="E276:G276"/>
-    <mergeCell ref="E1031:G1031"/>
+    <mergeCell ref="D1050:G1050"/>
     <mergeCell ref="A916:G916"/>
-    <mergeCell ref="D1050:G1050"/>
     <mergeCell ref="A1052:C1052"/>
     <mergeCell ref="E36:G36"/>
     <mergeCell ref="A970:C970"/>
@@ -13547,7 +13993,6 @@
     <mergeCell ref="D863:G863"/>
     <mergeCell ref="E718:G718"/>
     <mergeCell ref="A263:G263"/>
-    <mergeCell ref="E155:G155"/>
     <mergeCell ref="E760:G760"/>
     <mergeCell ref="A265:G265"/>
     <mergeCell ref="A563:G563"/>
@@ -13555,6 +14000,7 @@
     <mergeCell ref="A950:C950"/>
     <mergeCell ref="A195:C195"/>
     <mergeCell ref="D54:G54"/>
+    <mergeCell ref="E157:G157"/>
     <mergeCell ref="A116:C116"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="E949:G949"/>
@@ -13575,6 +14021,7 @@
     <mergeCell ref="A991:C991"/>
     <mergeCell ref="A398:G398"/>
     <mergeCell ref="D695:G695"/>
+    <mergeCell ref="E515:G515"/>
     <mergeCell ref="E175:G175"/>
     <mergeCell ref="A543:G543"/>
     <mergeCell ref="E337:G337"/>
@@ -13599,7 +14046,6 @@
     <mergeCell ref="D174:G174"/>
     <mergeCell ref="E1032:G1032"/>
     <mergeCell ref="E886:G886"/>
-    <mergeCell ref="A442:G442"/>
     <mergeCell ref="A727:G727"/>
     <mergeCell ref="E592:G592"/>
     <mergeCell ref="A844:C844"/>
@@ -13609,7 +14055,7 @@
     <mergeCell ref="A935:G935"/>
     <mergeCell ref="A145:G145"/>
     <mergeCell ref="A1027:G1027"/>
-    <mergeCell ref="D134:G134"/>
+    <mergeCell ref="A443:G443"/>
     <mergeCell ref="A704:G704"/>
     <mergeCell ref="A875:G875"/>
     <mergeCell ref="A196:C196"/>
@@ -13644,6 +14090,7 @@
     <mergeCell ref="E358:G358"/>
     <mergeCell ref="E971:G971"/>
     <mergeCell ref="A865:C865"/>
+    <mergeCell ref="E137:G137"/>
     <mergeCell ref="A872:G872"/>
     <mergeCell ref="A425:C425"/>
     <mergeCell ref="E1071:G1071"/>
@@ -13654,12 +14101,12 @@
     <mergeCell ref="A966:G966"/>
     <mergeCell ref="D315:G315"/>
     <mergeCell ref="A186:G186"/>
-    <mergeCell ref="A135:C135"/>
     <mergeCell ref="D800:G800"/>
     <mergeCell ref="A802:C802"/>
     <mergeCell ref="A491:C491"/>
     <mergeCell ref="A707:G707"/>
     <mergeCell ref="D379:G379"/>
+    <mergeCell ref="A511:G511"/>
     <mergeCell ref="A809:G809"/>
     <mergeCell ref="A980:G980"/>
     <mergeCell ref="A486:G486"/>
@@ -13698,6 +14145,7 @@
     <mergeCell ref="A283:G283"/>
     <mergeCell ref="A388:G388"/>
     <mergeCell ref="A746:G746"/>
+    <mergeCell ref="D514:G514"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A1102:G1102"/>
     <mergeCell ref="A296:C296"/>
@@ -13708,16 +14156,14 @@
     <mergeCell ref="A532:C532"/>
     <mergeCell ref="A306:G306"/>
     <mergeCell ref="D274:G274"/>
-    <mergeCell ref="D445:G445"/>
+    <mergeCell ref="E990:G990"/>
     <mergeCell ref="E928:G928"/>
-    <mergeCell ref="E990:G990"/>
     <mergeCell ref="A85:G85"/>
     <mergeCell ref="A634:C634"/>
     <mergeCell ref="E927:G927"/>
     <mergeCell ref="A893:G893"/>
-    <mergeCell ref="D511:G511"/>
+    <mergeCell ref="A1092:C1092"/>
     <mergeCell ref="A823:C823"/>
-    <mergeCell ref="A1092:C1092"/>
     <mergeCell ref="E95:G95"/>
     <mergeCell ref="E1092:G1092"/>
     <mergeCell ref="A143:G143"/>
@@ -13729,16 +14175,15 @@
     <mergeCell ref="A696:C696"/>
     <mergeCell ref="A225:G225"/>
     <mergeCell ref="A612:C612"/>
-    <mergeCell ref="A155:C155"/>
+    <mergeCell ref="A728:G728"/>
     <mergeCell ref="D571:G571"/>
-    <mergeCell ref="A728:G728"/>
     <mergeCell ref="A271:G271"/>
     <mergeCell ref="A1001:G1001"/>
     <mergeCell ref="A633:C633"/>
     <mergeCell ref="A676:C676"/>
+    <mergeCell ref="A157:C157"/>
     <mergeCell ref="A978:G978"/>
     <mergeCell ref="E215:G215"/>
-    <mergeCell ref="E513:G513"/>
     <mergeCell ref="E780:G780"/>
     <mergeCell ref="E402:G402"/>
     <mergeCell ref="A881:G881"/>
@@ -13750,6 +14195,7 @@
     <mergeCell ref="A454:G454"/>
     <mergeCell ref="E490:G490"/>
     <mergeCell ref="A818:G818"/>
+    <mergeCell ref="A515:C515"/>
     <mergeCell ref="A981:G981"/>
     <mergeCell ref="A175:C175"/>
     <mergeCell ref="A1041:G1041"/>
@@ -13777,7 +14223,6 @@
     <mergeCell ref="A902:G902"/>
     <mergeCell ref="A185:G185"/>
     <mergeCell ref="E1011:G1011"/>
-    <mergeCell ref="A508:G508"/>
     <mergeCell ref="A312:G312"/>
     <mergeCell ref="A106:G106"/>
     <mergeCell ref="A236:C236"/>
@@ -13789,6 +14234,8 @@
     <mergeCell ref="E216:G216"/>
     <mergeCell ref="E116:G116"/>
     <mergeCell ref="A1062:G1062"/>
+    <mergeCell ref="E516:G516"/>
+    <mergeCell ref="A132:G132"/>
     <mergeCell ref="A176:C176"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A223:G223"/>
@@ -13800,13 +14247,13 @@
     <mergeCell ref="A125:G125"/>
     <mergeCell ref="E275:G275"/>
     <mergeCell ref="A348:G348"/>
-    <mergeCell ref="E446:G446"/>
     <mergeCell ref="A923:G923"/>
     <mergeCell ref="A839:G839"/>
     <mergeCell ref="A347:G347"/>
     <mergeCell ref="A412:G412"/>
     <mergeCell ref="D551:G551"/>
     <mergeCell ref="A854:G854"/>
+    <mergeCell ref="E448:G448"/>
     <mergeCell ref="D467:G467"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A191:G191"/>

</xml_diff>

<commit_message>
Add 2 more children to Bằng Gà list
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -1537,14 +1537,14 @@
         </is>
       </c>
       <c r="F28" s="39" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G28" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H28" s="40" t="inlineStr">
         <is>
-          <t>✅ Đủ DS</t>
+          <t>⚠️ Vượt 2</t>
         </is>
       </c>
     </row>
@@ -7676,47 +7676,113 @@
       </c>
     </row>
     <row r="486" ht="16" customHeight="1">
-      <c r="A486" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 05 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="487" ht="8" customHeight="1"/>
-    <row r="488" ht="8" customHeight="1"/>
+      <c r="A486" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B486" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Thị Minh Anh</t>
+        </is>
+      </c>
+      <c r="C486" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 3A1 - TH&amp;THCS Trường Sơn</t>
+        </is>
+      </c>
+      <c r="D486" s="21" t="inlineStr">
+        <is>
+          <t>Bằng Gà</t>
+        </is>
+      </c>
+      <c r="E486" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F486" s="21" t="n"/>
+      <c r="G486" s="22" t="inlineStr">
+        <is>
+          <t>SN: 27/01/2017</t>
+        </is>
+      </c>
+    </row>
+    <row r="487" ht="8" customHeight="1">
+      <c r="A487" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B487" s="19" t="inlineStr">
+        <is>
+          <t>Bùi Quang Sáng</t>
+        </is>
+      </c>
+      <c r="C487" s="20" t="inlineStr">
+        <is>
+          <t>Mẫu giáo 5 tuổi - MN Trường Sơn</t>
+        </is>
+      </c>
+      <c r="D487" s="21" t="inlineStr">
+        <is>
+          <t>Bằng Gà</t>
+        </is>
+      </c>
+      <c r="E487" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F487" s="21" t="n"/>
+      <c r="G487" s="22" t="inlineStr">
+        <is>
+          <t>SN: 15/06/2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="488" ht="8" customHeight="1">
+      <c r="A488" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 07 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="489" ht="16" customHeight="1">
-      <c r="D489" s="24" t="inlineStr">
+      <c r="D489" s="24" t="n"/>
+    </row>
+    <row r="490" ht="18" customHeight="1">
+      <c r="A490" s="25" t="n"/>
+      <c r="E490" s="25" t="n"/>
+    </row>
+    <row r="491" ht="16" customHeight="1">
+      <c r="A491" s="26" t="n"/>
+      <c r="D491" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="490" ht="18" customHeight="1">
-      <c r="A490" s="25" t="inlineStr">
+    <row r="492" ht="6" customHeight="1">
+      <c r="A492" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E490" s="25" t="inlineStr">
+      <c r="E492" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="491" ht="16" customHeight="1">
-      <c r="A491" s="26" t="inlineStr">
+    <row r="493" ht="6" customHeight="1">
+      <c r="A493" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E491" s="26" t="inlineStr">
+      <c r="E493" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="492" ht="6" customHeight="1"/>
-    <row r="493" ht="6" customHeight="1"/>
     <row r="494" ht="6" customHeight="1"/>
     <row r="495" ht="4" customHeight="1">
       <c r="A495" s="27" t="n"/>
@@ -13815,12 +13881,14 @@
     <mergeCell ref="A1082:G1082"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="D1010:G1010"/>
+    <mergeCell ref="D491:G491"/>
     <mergeCell ref="A479:G479"/>
     <mergeCell ref="A650:G650"/>
     <mergeCell ref="D114:G114"/>
     <mergeCell ref="A665:G665"/>
     <mergeCell ref="A55:C55"/>
     <mergeCell ref="E717:G717"/>
+    <mergeCell ref="E492:G492"/>
     <mergeCell ref="E296:G296"/>
     <mergeCell ref="E738:G738"/>
     <mergeCell ref="A83:G83"/>
@@ -13838,7 +13906,6 @@
     <mergeCell ref="A643:G643"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="D1030:G1030"/>
-    <mergeCell ref="D489:G489"/>
     <mergeCell ref="E195:G195"/>
     <mergeCell ref="A358:C358"/>
     <mergeCell ref="D135:G135"/>
@@ -13859,7 +13926,6 @@
     <mergeCell ref="D1112:G1112"/>
     <mergeCell ref="D1091:G1091"/>
     <mergeCell ref="E675:G675"/>
-    <mergeCell ref="A490:C490"/>
     <mergeCell ref="E297:G297"/>
     <mergeCell ref="D194:G194"/>
     <mergeCell ref="E235:G235"/>
@@ -13933,7 +13999,6 @@
     <mergeCell ref="E697:G697"/>
     <mergeCell ref="E802:G802"/>
     <mergeCell ref="A71:G71"/>
-    <mergeCell ref="E491:G491"/>
     <mergeCell ref="A307:G307"/>
     <mergeCell ref="A641:G641"/>
     <mergeCell ref="E739:G739"/>
@@ -13961,6 +14026,7 @@
     <mergeCell ref="A522:G522"/>
     <mergeCell ref="A326:G326"/>
     <mergeCell ref="A1011:C1011"/>
+    <mergeCell ref="A492:C492"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="D926:G926"/>
@@ -14034,6 +14100,7 @@
     <mergeCell ref="A469:C469"/>
     <mergeCell ref="A622:G622"/>
     <mergeCell ref="A853:G853"/>
+    <mergeCell ref="A493:C493"/>
     <mergeCell ref="A945:G945"/>
     <mergeCell ref="A297:C297"/>
     <mergeCell ref="D884:G884"/>
@@ -14103,13 +14170,11 @@
     <mergeCell ref="A186:G186"/>
     <mergeCell ref="D800:G800"/>
     <mergeCell ref="A802:C802"/>
-    <mergeCell ref="A491:C491"/>
     <mergeCell ref="A707:G707"/>
     <mergeCell ref="D379:G379"/>
     <mergeCell ref="A511:G511"/>
     <mergeCell ref="A809:G809"/>
     <mergeCell ref="A980:G980"/>
-    <mergeCell ref="A486:G486"/>
     <mergeCell ref="A146:G146"/>
     <mergeCell ref="E255:G255"/>
     <mergeCell ref="E907:G907"/>
@@ -14193,7 +14258,6 @@
     <mergeCell ref="A91:G91"/>
     <mergeCell ref="A327:G327"/>
     <mergeCell ref="A454:G454"/>
-    <mergeCell ref="E490:G490"/>
     <mergeCell ref="A818:G818"/>
     <mergeCell ref="A515:C515"/>
     <mergeCell ref="A981:G981"/>
@@ -14208,6 +14272,7 @@
     <mergeCell ref="E572:G572"/>
     <mergeCell ref="A457:G457"/>
     <mergeCell ref="A906:C906"/>
+    <mergeCell ref="E493:G493"/>
     <mergeCell ref="A971:C971"/>
     <mergeCell ref="E553:G553"/>
     <mergeCell ref="E96:G96"/>
@@ -14236,6 +14301,7 @@
     <mergeCell ref="A1062:G1062"/>
     <mergeCell ref="E516:G516"/>
     <mergeCell ref="A132:G132"/>
+    <mergeCell ref="A488:G488"/>
     <mergeCell ref="A176:C176"/>
     <mergeCell ref="A25:G25"/>
     <mergeCell ref="A223:G223"/>

</xml_diff>

<commit_message>
Update Tiểu khu 6 and Tiểu khu 12 to 6 children each with school/grade
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -909,14 +909,14 @@
       </c>
       <c r="E8" s="8" t="inlineStr"/>
       <c r="F8" s="41" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G8" s="41" t="n">
         <v>0</v>
       </c>
       <c r="H8" s="42" t="inlineStr">
         <is>
-          <t>✅ Đủ DS</t>
+          <t>⚠️ Vượt 3</t>
         </is>
       </c>
     </row>
@@ -1033,14 +1033,14 @@
       </c>
       <c r="E12" s="8" t="inlineStr"/>
       <c r="F12" s="39" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G12" s="39" t="n">
         <v>0</v>
       </c>
       <c r="H12" s="40" t="inlineStr">
         <is>
-          <t>⚠️ Vượt 1</t>
+          <t>⚠️ Vượt 3</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3199,11 @@
           <t>Đỗ Gia Hưng</t>
         </is>
       </c>
-      <c r="C68" s="30" t="inlineStr"/>
+      <c r="C68" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 1</t>
+        </is>
+      </c>
       <c r="D68" s="31" t="inlineStr">
         <is>
           <t>Tiểu khu 6</t>
@@ -3226,7 +3230,11 @@
           <t>Nguyễn Phú Bảo Ngọc</t>
         </is>
       </c>
-      <c r="C69" s="30" t="inlineStr"/>
+      <c r="C69" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 8</t>
+        </is>
+      </c>
       <c r="D69" s="31" t="inlineStr">
         <is>
           <t>Tiểu khu 6</t>
@@ -3272,48 +3280,144 @@
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 03 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="8" customHeight="1"/>
-    <row r="73" ht="8" customHeight="1"/>
+      <c r="A71" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="B71" s="29" t="inlineStr">
+        <is>
+          <t>Lê Thảo Dương</t>
+        </is>
+      </c>
+      <c r="C71" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 7</t>
+        </is>
+      </c>
+      <c r="D71" s="31" t="inlineStr">
+        <is>
+          <t>Tiểu khu 6</t>
+        </is>
+      </c>
+      <c r="E71" s="30" t="inlineStr">
+        <is>
+          <t>Hoàn cảnh khó khăn</t>
+        </is>
+      </c>
+      <c r="F71" s="31" t="n"/>
+      <c r="G71" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="8" customHeight="1">
+      <c r="A72" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="B72" s="29" t="inlineStr">
+        <is>
+          <t>Nguyễn Tuấn Tú</t>
+        </is>
+      </c>
+      <c r="C72" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 8</t>
+        </is>
+      </c>
+      <c r="D72" s="31" t="inlineStr">
+        <is>
+          <t>Tiểu khu 6</t>
+        </is>
+      </c>
+      <c r="E72" s="30" t="inlineStr">
+        <is>
+          <t>Hoàn cảnh khó khăn</t>
+        </is>
+      </c>
+      <c r="F72" s="31" t="n"/>
+      <c r="G72" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="8" customHeight="1">
+      <c r="A73" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="B73" s="29" t="inlineStr">
+        <is>
+          <t>Nguyễn Thị Bảo Ngọc</t>
+        </is>
+      </c>
+      <c r="C73" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 5</t>
+        </is>
+      </c>
+      <c r="D73" s="31" t="inlineStr">
+        <is>
+          <t>Tiểu khu 6</t>
+        </is>
+      </c>
+      <c r="E73" s="30" t="inlineStr">
+        <is>
+          <t>Bố mẹ bỏ nhau, ở với ông bà, hoàn cảnh khó khăn</t>
+        </is>
+      </c>
+      <c r="F73" s="31" t="n"/>
+      <c r="G73" s="32" t="inlineStr">
+        <is>
+          <t>SN: 2015</t>
+        </is>
+      </c>
+    </row>
     <row r="74" ht="16" customHeight="1">
-      <c r="D74" s="24" t="inlineStr">
+      <c r="A74" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 06 trẻ em.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="25" t="n"/>
+      <c r="E75" s="25" t="n"/>
+    </row>
+    <row r="76" ht="16" customHeight="1">
+      <c r="A76" s="26" t="n"/>
+      <c r="E76" s="26" t="n"/>
+    </row>
+    <row r="77" ht="6" customHeight="1">
+      <c r="D77" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="25" t="inlineStr">
+    <row r="78" ht="6" customHeight="1">
+      <c r="A78" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E75" s="25" t="inlineStr">
+      <c r="E78" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="16" customHeight="1">
-      <c r="A76" s="26" t="inlineStr">
+    <row r="79" ht="6" customHeight="1">
+      <c r="A79" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E76" s="26" t="inlineStr">
+      <c r="E79" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="6" customHeight="1"/>
-    <row r="78" ht="6" customHeight="1"/>
-    <row r="79" ht="6" customHeight="1"/>
     <row r="80" ht="4" customHeight="1">
       <c r="A80" s="27" t="n"/>
       <c r="B80" s="27" t="n"/>
@@ -4082,7 +4186,7 @@
       </c>
       <c r="C148" s="20" t="inlineStr">
         <is>
-          <t>Mầm non</t>
+          <t>Mẫu giáo 5 tuổi - Trường Liên Cơ</t>
         </is>
       </c>
       <c r="D148" s="21" t="inlineStr">
@@ -4113,7 +4217,7 @@
       </c>
       <c r="C149" s="20" t="inlineStr">
         <is>
-          <t>Lớp 5</t>
+          <t>Lớp 5 - TH&amp;THCS Cửu Long</t>
         </is>
       </c>
       <c r="D149" s="21" t="inlineStr">
@@ -4144,7 +4248,7 @@
       </c>
       <c r="C150" s="20" t="inlineStr">
         <is>
-          <t>Lớp 7</t>
+          <t>Lớp 7 - TH&amp;THCS Cửu Long</t>
         </is>
       </c>
       <c r="D150" s="21" t="inlineStr">
@@ -4192,50 +4296,111 @@
       </c>
     </row>
     <row r="152" ht="8" customHeight="1">
-      <c r="A152" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 04 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="8" customHeight="1"/>
+      <c r="A152" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B152" s="19" t="inlineStr">
+        <is>
+          <t>Trần Huyền Trang</t>
+        </is>
+      </c>
+      <c r="C152" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 6 - TH&amp;THCS Cửu Long</t>
+        </is>
+      </c>
+      <c r="D152" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu 12</t>
+        </is>
+      </c>
+      <c r="E152" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F152" s="21" t="n"/>
+      <c r="G152" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="8" customHeight="1">
+      <c r="A153" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B153" s="19" t="inlineStr">
+        <is>
+          <t>Trương Bảo Nam</t>
+        </is>
+      </c>
+      <c r="C153" s="20" t="inlineStr"/>
+      <c r="D153" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu 12</t>
+        </is>
+      </c>
+      <c r="E153" s="20" t="inlineStr">
+        <is>
+          <t>Không có bố, bị thận bẩm sinh</t>
+        </is>
+      </c>
+      <c r="F153" s="21" t="n"/>
+      <c r="G153" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2023</t>
+        </is>
+      </c>
+    </row>
     <row r="154" ht="16" customHeight="1">
-      <c r="D154" s="24" t="n"/>
+      <c r="A154" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 06 trẻ em.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="18" customHeight="1">
       <c r="A155" s="25" t="n"/>
-      <c r="D155" s="24" t="inlineStr">
+      <c r="D155" s="24" t="n"/>
+    </row>
+    <row r="156" ht="16" customHeight="1">
+      <c r="A156" s="25" t="n"/>
+      <c r="D156" s="24" t="n"/>
+      <c r="E156" s="25" t="n"/>
+    </row>
+    <row r="157" ht="6" customHeight="1">
+      <c r="A157" s="25" t="n"/>
+      <c r="D157" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="16" customHeight="1">
-      <c r="A156" s="25" t="inlineStr">
+    <row r="158" ht="6" customHeight="1">
+      <c r="A158" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E156" s="25" t="inlineStr">
+      <c r="E158" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="157" ht="6" customHeight="1">
-      <c r="A157" s="26" t="inlineStr">
+    <row r="159" ht="6" customHeight="1">
+      <c r="A159" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E157" s="26" t="inlineStr">
+      <c r="E159" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="158" ht="6" customHeight="1"/>
-    <row r="159" ht="6" customHeight="1"/>
     <row r="160" ht="4" customHeight="1">
       <c r="A160" s="27" t="n"/>
       <c r="B160" s="27" t="n"/>
@@ -13858,7 +14023,6 @@
     <mergeCell ref="A255:C255"/>
     <mergeCell ref="A725:G725"/>
     <mergeCell ref="A231:G231"/>
-    <mergeCell ref="D74:G74"/>
     <mergeCell ref="A206:G206"/>
     <mergeCell ref="A655:C655"/>
     <mergeCell ref="A333:G333"/>
@@ -13930,6 +14094,7 @@
     <mergeCell ref="D194:G194"/>
     <mergeCell ref="E235:G235"/>
     <mergeCell ref="E533:G533"/>
+    <mergeCell ref="A79:C79"/>
     <mergeCell ref="E676:G676"/>
     <mergeCell ref="A749:G749"/>
     <mergeCell ref="A434:G434"/>
@@ -13945,10 +14110,8 @@
     <mergeCell ref="A1093:C1093"/>
     <mergeCell ref="A671:G671"/>
     <mergeCell ref="A381:C381"/>
-    <mergeCell ref="A152:G152"/>
     <mergeCell ref="D14:G14"/>
     <mergeCell ref="A686:G686"/>
-    <mergeCell ref="A76:C76"/>
     <mergeCell ref="E844:G844"/>
     <mergeCell ref="A226:G226"/>
     <mergeCell ref="E196:G196"/>
@@ -13961,6 +14124,7 @@
     <mergeCell ref="A928:C928"/>
     <mergeCell ref="A286:G286"/>
     <mergeCell ref="A528:G528"/>
+    <mergeCell ref="A74:G74"/>
     <mergeCell ref="A851:G851"/>
     <mergeCell ref="A1022:G1022"/>
     <mergeCell ref="A216:C216"/>
@@ -13982,7 +14146,6 @@
     <mergeCell ref="A613:C613"/>
     <mergeCell ref="A45:G45"/>
     <mergeCell ref="A1042:G1042"/>
-    <mergeCell ref="D155:G155"/>
     <mergeCell ref="A623:G623"/>
     <mergeCell ref="A523:G523"/>
     <mergeCell ref="A345:G345"/>
@@ -13998,7 +14161,6 @@
     <mergeCell ref="E35:G35"/>
     <mergeCell ref="E697:G697"/>
     <mergeCell ref="E802:G802"/>
-    <mergeCell ref="A71:G71"/>
     <mergeCell ref="A307:G307"/>
     <mergeCell ref="A641:G641"/>
     <mergeCell ref="E739:G739"/>
@@ -14013,6 +14175,7 @@
     <mergeCell ref="A811:G811"/>
     <mergeCell ref="A1109:G1109"/>
     <mergeCell ref="A769:G769"/>
+    <mergeCell ref="A159:C159"/>
     <mergeCell ref="E359:G359"/>
     <mergeCell ref="A759:C759"/>
     <mergeCell ref="D34:G34"/>
@@ -14055,7 +14218,6 @@
     <mergeCell ref="A683:G683"/>
     <mergeCell ref="D1070:G1070"/>
     <mergeCell ref="D336:G336"/>
-    <mergeCell ref="E156:G156"/>
     <mergeCell ref="D863:G863"/>
     <mergeCell ref="E718:G718"/>
     <mergeCell ref="A263:G263"/>
@@ -14066,7 +14228,6 @@
     <mergeCell ref="A950:C950"/>
     <mergeCell ref="A195:C195"/>
     <mergeCell ref="D54:G54"/>
-    <mergeCell ref="E157:G157"/>
     <mergeCell ref="A116:C116"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="E949:G949"/>
@@ -14081,7 +14242,6 @@
     <mergeCell ref="A1067:G1067"/>
     <mergeCell ref="D758:G758"/>
     <mergeCell ref="A917:G917"/>
-    <mergeCell ref="E75:G75"/>
     <mergeCell ref="E1072:G1072"/>
     <mergeCell ref="E317:G317"/>
     <mergeCell ref="A991:C991"/>
@@ -14130,6 +14290,7 @@
     <mergeCell ref="D357:G357"/>
     <mergeCell ref="A203:G203"/>
     <mergeCell ref="A717:C717"/>
+    <mergeCell ref="E78:G78"/>
     <mergeCell ref="E176:G176"/>
     <mergeCell ref="E447:G447"/>
     <mergeCell ref="A654:C654"/>
@@ -14152,6 +14313,7 @@
     <mergeCell ref="A275:C275"/>
     <mergeCell ref="D716:G716"/>
     <mergeCell ref="A369:G369"/>
+    <mergeCell ref="E79:G79"/>
     <mergeCell ref="A748:G748"/>
     <mergeCell ref="E613:G613"/>
     <mergeCell ref="E358:G358"/>
@@ -14159,6 +14321,7 @@
     <mergeCell ref="A865:C865"/>
     <mergeCell ref="E137:G137"/>
     <mergeCell ref="A872:G872"/>
+    <mergeCell ref="A158:C158"/>
     <mergeCell ref="A425:C425"/>
     <mergeCell ref="E1071:G1071"/>
     <mergeCell ref="A432:G432"/>
@@ -14199,7 +14362,6 @@
     <mergeCell ref="E316:G316"/>
     <mergeCell ref="E552:G552"/>
     <mergeCell ref="A886:C886"/>
-    <mergeCell ref="E76:G76"/>
     <mergeCell ref="E380:G380"/>
     <mergeCell ref="A580:G580"/>
     <mergeCell ref="D969:G969"/>
@@ -14212,6 +14374,7 @@
     <mergeCell ref="A746:G746"/>
     <mergeCell ref="D514:G514"/>
     <mergeCell ref="A36:C36"/>
+    <mergeCell ref="A154:G154"/>
     <mergeCell ref="A1102:G1102"/>
     <mergeCell ref="A296:C296"/>
     <mergeCell ref="A285:G285"/>
@@ -14223,9 +14386,11 @@
     <mergeCell ref="D274:G274"/>
     <mergeCell ref="E990:G990"/>
     <mergeCell ref="E928:G928"/>
+    <mergeCell ref="A78:C78"/>
     <mergeCell ref="A85:G85"/>
     <mergeCell ref="A634:C634"/>
     <mergeCell ref="E927:G927"/>
+    <mergeCell ref="E158:G158"/>
     <mergeCell ref="A893:G893"/>
     <mergeCell ref="A1092:C1092"/>
     <mergeCell ref="A823:C823"/>
@@ -14235,7 +14400,6 @@
     <mergeCell ref="A603:G603"/>
     <mergeCell ref="A937:G937"/>
     <mergeCell ref="A11:G11"/>
-    <mergeCell ref="A156:C156"/>
     <mergeCell ref="D821:G821"/>
     <mergeCell ref="A696:C696"/>
     <mergeCell ref="A225:G225"/>
@@ -14244,15 +14408,14 @@
     <mergeCell ref="D571:G571"/>
     <mergeCell ref="A271:G271"/>
     <mergeCell ref="A1001:G1001"/>
+    <mergeCell ref="D77:G77"/>
     <mergeCell ref="A633:C633"/>
     <mergeCell ref="A676:C676"/>
-    <mergeCell ref="A157:C157"/>
     <mergeCell ref="A978:G978"/>
     <mergeCell ref="E215:G215"/>
     <mergeCell ref="E780:G780"/>
     <mergeCell ref="E402:G402"/>
     <mergeCell ref="A881:G881"/>
-    <mergeCell ref="A75:C75"/>
     <mergeCell ref="A1072:C1072"/>
     <mergeCell ref="A317:C317"/>
     <mergeCell ref="A91:G91"/>
@@ -14268,6 +14431,7 @@
     <mergeCell ref="A1113:C1113"/>
     <mergeCell ref="A520:G520"/>
     <mergeCell ref="A907:C907"/>
+    <mergeCell ref="E159:G159"/>
     <mergeCell ref="D611:G611"/>
     <mergeCell ref="E572:G572"/>
     <mergeCell ref="A457:G457"/>
@@ -14310,6 +14474,7 @@
     <mergeCell ref="A1061:G1061"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="E236:G236"/>
+    <mergeCell ref="D157:G157"/>
     <mergeCell ref="A125:G125"/>
     <mergeCell ref="E275:G275"/>
     <mergeCell ref="A348:G348"/>

</xml_diff>

<commit_message>
Update Tiểu khu Mò to 5 children with school/grade
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -1191,14 +1191,14 @@
         </is>
       </c>
       <c r="F17" s="39" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G17" s="39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H17" s="40" t="inlineStr">
         <is>
-          <t>⏳ Còn thiếu 2</t>
+          <t>⚠️ Vượt 2</t>
         </is>
       </c>
     </row>
@@ -5268,12 +5268,12 @@
       </c>
       <c r="B248" s="19" t="inlineStr">
         <is>
-          <t>Đinh Quỳnh Như</t>
+          <t>Hoàng Văn Minh</t>
         </is>
       </c>
       <c r="C248" s="20" t="inlineStr">
         <is>
-          <t>Lớp 5 - TH&amp;THCS Hùng Sơn</t>
+          <t>Lớp 3A3 - TH&amp;THCS Hùng Sơn</t>
         </is>
       </c>
       <c r="D248" s="21" t="inlineStr">
@@ -5283,28 +5283,36 @@
       </c>
       <c r="E248" s="20" t="inlineStr">
         <is>
-          <t>Hộ cận nghèo đơn thân, mẹ bệnh tật không có việc làm, cháu là TEKT</t>
+          <t>Hộ khó khăn</t>
         </is>
       </c>
       <c r="F248" s="21" t="inlineStr"/>
-      <c r="G248" s="22" t="inlineStr">
-        <is>
-          <t>SN: 21/01/2015</t>
-        </is>
-      </c>
+      <c r="G248" s="22" t="inlineStr"/>
     </row>
     <row r="249" ht="22" customHeight="1">
       <c r="A249" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B249" s="19" t="inlineStr"/>
-      <c r="C249" s="20" t="inlineStr"/>
+      <c r="B249" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Khánh Chi</t>
+        </is>
+      </c>
+      <c r="C249" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 7A2 - TH&amp;THCS Cửu Long</t>
+        </is>
+      </c>
       <c r="D249" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu Mò</t>
         </is>
       </c>
-      <c r="E249" s="20" t="inlineStr"/>
+      <c r="E249" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F249" s="21" t="inlineStr"/>
       <c r="G249" s="22" t="inlineStr"/>
     </row>
@@ -5312,59 +5320,133 @@
       <c r="A250" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B250" s="19" t="inlineStr"/>
-      <c r="C250" s="20" t="inlineStr"/>
+      <c r="B250" s="19" t="inlineStr">
+        <is>
+          <t>Nguyễn Phương Nhi</t>
+        </is>
+      </c>
+      <c r="C250" s="20" t="inlineStr">
+        <is>
+          <t>Mẫu giáo 5 tuổi - MN Liên Cơ</t>
+        </is>
+      </c>
       <c r="D250" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu Mò</t>
         </is>
       </c>
-      <c r="E250" s="20" t="inlineStr"/>
+      <c r="E250" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F250" s="21" t="inlineStr"/>
       <c r="G250" s="22" t="inlineStr"/>
     </row>
     <row r="251" ht="16" customHeight="1">
-      <c r="A251" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 03 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="252" ht="8" customHeight="1"/>
-    <row r="253" ht="8" customHeight="1"/>
+      <c r="A251" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="B251" s="19" t="inlineStr">
+        <is>
+          <t>Đinh Khánh Ngân</t>
+        </is>
+      </c>
+      <c r="C251" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 8A3 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
+      <c r="D251" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu Mò</t>
+        </is>
+      </c>
+      <c r="E251" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F251" s="21" t="n"/>
+      <c r="G251" s="22" t="inlineStr"/>
+    </row>
+    <row r="252" ht="8" customHeight="1">
+      <c r="A252" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B252" s="19" t="inlineStr">
+        <is>
+          <t>Đinh Quỳnh Như</t>
+        </is>
+      </c>
+      <c r="C252" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Hùng Sơn</t>
+        </is>
+      </c>
+      <c r="D252" s="21" t="inlineStr">
+        <is>
+          <t>Tiểu khu Mò</t>
+        </is>
+      </c>
+      <c r="E252" s="20" t="inlineStr">
+        <is>
+          <t>Hộ cận nghèo đơn thân, mẹ bệnh tật không có việc làm, cháu là TEKT</t>
+        </is>
+      </c>
+      <c r="F252" s="21" t="n"/>
+      <c r="G252" s="22" t="inlineStr">
+        <is>
+          <t>SN: 21/01/2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="253" ht="8" customHeight="1">
+      <c r="A253" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 05 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="254" ht="16" customHeight="1">
-      <c r="D254" s="24" t="inlineStr">
+      <c r="D254" s="24" t="n"/>
+    </row>
+    <row r="255" ht="18" customHeight="1">
+      <c r="A255" s="25" t="n"/>
+      <c r="E255" s="25" t="n"/>
+    </row>
+    <row r="256" ht="16" customHeight="1">
+      <c r="A256" s="26" t="n"/>
+      <c r="D256" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="255" ht="18" customHeight="1">
-      <c r="A255" s="25" t="inlineStr">
+    <row r="257" ht="6" customHeight="1">
+      <c r="A257" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E255" s="25" t="inlineStr">
+      <c r="E257" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="256" ht="16" customHeight="1">
-      <c r="A256" s="26" t="inlineStr">
+    <row r="258" ht="6" customHeight="1">
+      <c r="A258" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E256" s="26" t="inlineStr">
+      <c r="E258" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="257" ht="6" customHeight="1"/>
-    <row r="258" ht="6" customHeight="1"/>
     <row r="259" ht="6" customHeight="1"/>
     <row r="260" ht="4" customHeight="1">
       <c r="A260" s="27" t="n"/>
@@ -14020,7 +14102,6 @@
     <row r="1119" ht="6" customHeight="1"/>
   </sheetData>
   <mergeCells count="486">
-    <mergeCell ref="A255:C255"/>
     <mergeCell ref="A725:G725"/>
     <mergeCell ref="A231:G231"/>
     <mergeCell ref="A206:G206"/>
@@ -14036,7 +14117,6 @@
     <mergeCell ref="A103:G103"/>
     <mergeCell ref="E16:G16"/>
     <mergeCell ref="E1052:G1052"/>
-    <mergeCell ref="D254:G254"/>
     <mergeCell ref="A413:G413"/>
     <mergeCell ref="A1071:C1071"/>
     <mergeCell ref="A776:G776"/>
@@ -14065,7 +14145,9 @@
     <mergeCell ref="A797:G797"/>
     <mergeCell ref="A812:G812"/>
     <mergeCell ref="A1039:G1039"/>
+    <mergeCell ref="A258:C258"/>
     <mergeCell ref="D674:G674"/>
+    <mergeCell ref="E258:G258"/>
     <mergeCell ref="A205:G205"/>
     <mergeCell ref="A643:G643"/>
     <mergeCell ref="A65:G65"/>
@@ -14111,11 +14193,11 @@
     <mergeCell ref="A671:G671"/>
     <mergeCell ref="A381:C381"/>
     <mergeCell ref="D14:G14"/>
+    <mergeCell ref="D256:G256"/>
     <mergeCell ref="A686:G686"/>
     <mergeCell ref="E844:G844"/>
     <mergeCell ref="A226:G226"/>
     <mergeCell ref="E196:G196"/>
-    <mergeCell ref="E256:G256"/>
     <mergeCell ref="E612:G612"/>
     <mergeCell ref="A501:G501"/>
     <mergeCell ref="A243:G243"/>
@@ -14138,6 +14220,7 @@
     <mergeCell ref="E338:G338"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="E1012:G1012"/>
+    <mergeCell ref="E257:G257"/>
     <mergeCell ref="A468:C468"/>
     <mergeCell ref="E865:G865"/>
     <mergeCell ref="A755:G755"/>
@@ -14252,9 +14335,9 @@
     <mergeCell ref="A543:G543"/>
     <mergeCell ref="E337:G337"/>
     <mergeCell ref="E573:G573"/>
-    <mergeCell ref="A251:G251"/>
     <mergeCell ref="E1113:G1113"/>
     <mergeCell ref="A126:G126"/>
+    <mergeCell ref="A253:G253"/>
     <mergeCell ref="A1079:G1079"/>
     <mergeCell ref="A324:G324"/>
     <mergeCell ref="A469:C469"/>
@@ -14286,7 +14369,6 @@
     <mergeCell ref="A704:G704"/>
     <mergeCell ref="A875:G875"/>
     <mergeCell ref="A196:C196"/>
-    <mergeCell ref="A256:C256"/>
     <mergeCell ref="D357:G357"/>
     <mergeCell ref="A203:G203"/>
     <mergeCell ref="A717:C717"/>
@@ -14309,6 +14391,7 @@
     <mergeCell ref="A354:G354"/>
     <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1012:C1012"/>
+    <mergeCell ref="A257:C257"/>
     <mergeCell ref="A1081:G1081"/>
     <mergeCell ref="A275:C275"/>
     <mergeCell ref="D716:G716"/>
@@ -14339,7 +14422,6 @@
     <mergeCell ref="A809:G809"/>
     <mergeCell ref="A980:G980"/>
     <mergeCell ref="A146:G146"/>
-    <mergeCell ref="E255:G255"/>
     <mergeCell ref="E907:G907"/>
     <mergeCell ref="A66:G66"/>
     <mergeCell ref="E759:G759"/>

</xml_diff>

<commit_message>
Add 2 children to Tiểu khu 4
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -879,14 +879,14 @@
       </c>
       <c r="E7" s="8" t="inlineStr"/>
       <c r="F7" s="41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G7" s="41" t="n">
         <v>0</v>
       </c>
       <c r="H7" s="42" t="inlineStr">
         <is>
-          <t>✅ Đủ DS</t>
+          <t>⚠️ Vượt 2</t>
         </is>
       </c>
     </row>
@@ -3071,47 +3071,113 @@
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="23" t="inlineStr">
-        <is>
-          <t>Ấn định danh sách có 03 trẻ em.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="8" customHeight="1"/>
-    <row r="53" ht="8" customHeight="1"/>
+      <c r="A51" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B51" s="29" t="inlineStr">
+        <is>
+          <t>Nguyễn Khánh Đông</t>
+        </is>
+      </c>
+      <c r="C51" s="30" t="inlineStr">
+        <is>
+          <t>Lớp 5 - TH&amp;THCS Bải Lạng</t>
+        </is>
+      </c>
+      <c r="D51" s="36" t="inlineStr">
+        <is>
+          <t>Tiểu khu 4</t>
+        </is>
+      </c>
+      <c r="E51" s="30" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F51" s="36" t="n"/>
+      <c r="G51" s="32" t="inlineStr">
+        <is>
+          <t>SN: 12/05/2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="8" customHeight="1">
+      <c r="A52" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="B52" s="29" t="inlineStr">
+        <is>
+          <t>Nguyễn Đức Huy</t>
+        </is>
+      </c>
+      <c r="C52" s="30" t="inlineStr">
+        <is>
+          <t>MN Cửu Long</t>
+        </is>
+      </c>
+      <c r="D52" s="36" t="inlineStr">
+        <is>
+          <t>Tiểu khu 4</t>
+        </is>
+      </c>
+      <c r="E52" s="30" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
+      <c r="F52" s="36" t="n"/>
+      <c r="G52" s="32" t="inlineStr">
+        <is>
+          <t>SN: 03/09/2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="8" customHeight="1">
+      <c r="A53" s="23" t="inlineStr">
+        <is>
+          <t>Ấn định danh sách có 05 trẻ em.</t>
+        </is>
+      </c>
+    </row>
     <row r="54" ht="16" customHeight="1">
-      <c r="D54" s="24" t="inlineStr">
+      <c r="D54" s="24" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="25" t="n"/>
+      <c r="E55" s="25" t="n"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="26" t="n"/>
+      <c r="D56" s="24" t="inlineStr">
         <is>
           <t>......., ngày .... tháng .... năm 2026</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="25" t="inlineStr">
+    <row r="57" ht="6" customHeight="1">
+      <c r="A57" s="25" t="inlineStr">
         <is>
           <t>NGƯỜI LẬP BIỂU</t>
         </is>
       </c>
-      <c r="E55" s="25" t="inlineStr">
+      <c r="E57" s="25" t="inlineStr">
         <is>
           <t>THỦ TRƯỞNG ĐƠN VỊ</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="26" t="inlineStr">
+    <row r="58" ht="6" customHeight="1">
+      <c r="A58" s="26" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ và tên)</t>
         </is>
       </c>
-      <c r="E56" s="26" t="inlineStr">
+      <c r="E58" s="26" t="inlineStr">
         <is>
           <t>(Ký tên, đóng dấu)</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="6" customHeight="1"/>
-    <row r="58" ht="6" customHeight="1"/>
     <row r="59" ht="6" customHeight="1"/>
     <row r="60" ht="4" customHeight="1">
       <c r="A60" s="27" t="n"/>
@@ -14108,6 +14174,7 @@
     <mergeCell ref="A655:C655"/>
     <mergeCell ref="A333:G333"/>
     <mergeCell ref="A136:C136"/>
+    <mergeCell ref="A57:C57"/>
     <mergeCell ref="A1000:G1000"/>
     <mergeCell ref="A245:G245"/>
     <mergeCell ref="A949:C949"/>
@@ -14125,12 +14192,12 @@
     <mergeCell ref="A1082:G1082"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="D1010:G1010"/>
+    <mergeCell ref="D56:G56"/>
     <mergeCell ref="D491:G491"/>
     <mergeCell ref="A479:G479"/>
     <mergeCell ref="A650:G650"/>
     <mergeCell ref="D114:G114"/>
     <mergeCell ref="A665:G665"/>
-    <mergeCell ref="A55:C55"/>
     <mergeCell ref="E717:G717"/>
     <mergeCell ref="E492:G492"/>
     <mergeCell ref="E296:G296"/>
@@ -14147,6 +14214,7 @@
     <mergeCell ref="A1039:G1039"/>
     <mergeCell ref="A258:C258"/>
     <mergeCell ref="D674:G674"/>
+    <mergeCell ref="A58:C58"/>
     <mergeCell ref="E258:G258"/>
     <mergeCell ref="A205:G205"/>
     <mergeCell ref="A643:G643"/>
@@ -14267,7 +14335,6 @@
     <mergeCell ref="D737:G737"/>
     <mergeCell ref="A96:C96"/>
     <mergeCell ref="E1051:G1051"/>
-    <mergeCell ref="E56:G56"/>
     <mergeCell ref="E906:G906"/>
     <mergeCell ref="A522:G522"/>
     <mergeCell ref="A326:G326"/>
@@ -14310,7 +14377,6 @@
     <mergeCell ref="A830:G830"/>
     <mergeCell ref="A950:C950"/>
     <mergeCell ref="A195:C195"/>
-    <mergeCell ref="D54:G54"/>
     <mergeCell ref="A116:C116"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="E949:G949"/>
@@ -14341,6 +14407,7 @@
     <mergeCell ref="A1079:G1079"/>
     <mergeCell ref="A324:G324"/>
     <mergeCell ref="A469:C469"/>
+    <mergeCell ref="A53:G53"/>
     <mergeCell ref="A622:G622"/>
     <mergeCell ref="A853:G853"/>
     <mergeCell ref="A493:C493"/>
@@ -14352,10 +14419,12 @@
     <mergeCell ref="A533:C533"/>
     <mergeCell ref="A111:G111"/>
     <mergeCell ref="E655:G655"/>
+    <mergeCell ref="E57:G57"/>
     <mergeCell ref="D423:G423"/>
     <mergeCell ref="D174:G174"/>
     <mergeCell ref="E1032:G1032"/>
     <mergeCell ref="E886:G886"/>
+    <mergeCell ref="E58:G58"/>
     <mergeCell ref="A727:G727"/>
     <mergeCell ref="E592:G592"/>
     <mergeCell ref="A844:C844"/>
@@ -14434,7 +14503,6 @@
     <mergeCell ref="A896:G896"/>
     <mergeCell ref="A420:G420"/>
     <mergeCell ref="A662:G662"/>
-    <mergeCell ref="A56:C56"/>
     <mergeCell ref="A960:G960"/>
     <mergeCell ref="A435:G435"/>
     <mergeCell ref="D94:G94"/>
@@ -14570,7 +14638,6 @@
     <mergeCell ref="D467:G467"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A191:G191"/>
-    <mergeCell ref="A51:G51"/>
     <mergeCell ref="A620:G620"/>
     <mergeCell ref="A115:C115"/>
     <mergeCell ref="A476:G476"/>
@@ -14582,7 +14649,6 @@
     <mergeCell ref="A337:C337"/>
     <mergeCell ref="A402:C402"/>
     <mergeCell ref="E1114:G1114"/>
-    <mergeCell ref="E55:G55"/>
     <mergeCell ref="E822:G822"/>
     <mergeCell ref="A781:C781"/>
     <mergeCell ref="D214:G214"/>

</xml_diff>

<commit_message>
Add 3 children to Tiểu khu 2
https://claude.ai/code/session_01VFxCZ9KmZkFz3zPeBX6EnK
</commit_message>
<xml_diff>
--- a/DS_Tang_Qua_Shinwon_2026_v3.xlsx
+++ b/DS_Tang_Qua_Shinwon_2026_v3.xlsx
@@ -819,14 +819,14 @@
         </is>
       </c>
       <c r="F5" s="39" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H5" s="40" t="inlineStr">
         <is>
-          <t>⏳ Còn thiếu 3</t>
+          <t>✅ Đủ DS</t>
         </is>
       </c>
     </row>
@@ -2603,46 +2603,94 @@
       <c r="A8" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="B8" s="19" t="inlineStr"/>
-      <c r="C8" s="20" t="inlineStr"/>
+      <c r="B8" s="19" t="inlineStr">
+        <is>
+          <t>Cao Bảo An</t>
+        </is>
+      </c>
+      <c r="C8" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 3</t>
+        </is>
+      </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 2</t>
         </is>
       </c>
-      <c r="E8" s="20" t="inlineStr"/>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F8" s="21" t="inlineStr"/>
-      <c r="G8" s="22" t="inlineStr"/>
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2017</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="B9" s="19" t="inlineStr"/>
-      <c r="C9" s="20" t="inlineStr"/>
+      <c r="B9" s="19" t="inlineStr">
+        <is>
+          <t>Trần Phương Quỳnh Chi</t>
+        </is>
+      </c>
+      <c r="C9" s="20" t="inlineStr">
+        <is>
+          <t>Lớp 5</t>
+        </is>
+      </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 2</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr"/>
+      <c r="E9" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F9" s="21" t="inlineStr"/>
-      <c r="G9" s="22" t="inlineStr"/>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2015</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="19" t="inlineStr"/>
-      <c r="C10" s="20" t="inlineStr"/>
+      <c r="B10" s="19" t="inlineStr">
+        <is>
+          <t>Trần Hoàng Việt</t>
+        </is>
+      </c>
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Mầm non</t>
+        </is>
+      </c>
       <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Tiểu khu 2</t>
         </is>
       </c>
-      <c r="E10" s="20" t="inlineStr"/>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Hộ khó khăn</t>
+        </is>
+      </c>
       <c r="F10" s="21" t="inlineStr"/>
-      <c r="G10" s="22" t="inlineStr"/>
+      <c r="G10" s="22" t="inlineStr">
+        <is>
+          <t>SN: 2020</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="23" t="inlineStr">

</xml_diff>